<commit_message>
feat(security): remove all institutional prefixes (COM, SBC, PRO) and genericize domain references
</commit_message>
<xml_diff>
--- a/ejemplo.xlsx
+++ b/ejemplo.xlsx
@@ -916,7 +916,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>COM PEREZ JUAN</t>
+          <t>PEREZ JUAN</t>
         </is>
       </c>
       <c r="B4" s="27" t="n"/>
@@ -956,7 +956,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>COM GONZALEZ MARIA</t>
+          <t>GONZALEZ MARIA</t>
         </is>
       </c>
       <c r="B5" s="27" t="n"/>
@@ -996,7 +996,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>COM SOTO CARLOS</t>
+          <t>SOTO CARLOS</t>
         </is>
       </c>
       <c r="B6" s="27" t="n"/>
@@ -1040,7 +1040,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>COM SILVA CLAUDIA</t>
+          <t>SILVA CLAUDIA</t>
         </is>
       </c>
       <c r="B7" s="27" t="n"/>
@@ -1080,7 +1080,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>COM ROJAS CECILIA</t>
+          <t>ROJAS CECILIA</t>
         </is>
       </c>
       <c r="B8" s="29" t="n"/>
@@ -1124,7 +1124,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>SBC DIAZ CATHERINE</t>
+          <t>DIAZ CATHERINE</t>
         </is>
       </c>
       <c r="B9" s="27" t="n"/>
@@ -1168,7 +1168,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>PRO MORALES JOSE</t>
+          <t>MORALES JOSE</t>
         </is>
       </c>
       <c r="B10" s="27" t="n"/>
@@ -1208,7 +1208,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>PRO ALVAREZ SUSANA</t>
+          <t>ALVAREZ SUSANA</t>
         </is>
       </c>
       <c r="B11" s="28" t="n"/>
@@ -1252,7 +1252,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>PRO CASTILLO PAMELA</t>
+          <t>CASTILLO PAMELA</t>
         </is>
       </c>
       <c r="B12" s="27" t="n"/>
@@ -1292,7 +1292,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>PRO TORRES PATRICIO</t>
+          <t>TORRES PATRICIO</t>
         </is>
       </c>
       <c r="B13" s="28" t="n"/>
@@ -1332,7 +1332,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>PRO TAPIA KARINA</t>
+          <t>TAPIA KARINA</t>
         </is>
       </c>
       <c r="B14" s="28" t="n"/>
@@ -1376,7 +1376,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>PRO CONTRERAS RODRIGO</t>
+          <t>CONTRERAS RODRIGO</t>
         </is>
       </c>
       <c r="B15" s="30" t="n"/>
@@ -1416,7 +1416,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>PRO FLORES CAMILA</t>
+          <t>FLORES CAMILA</t>
         </is>
       </c>
       <c r="B16" s="30" t="n"/>
@@ -1456,7 +1456,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>PRO NEIRA PRISCILA</t>
+          <t>NEIRA PRISCILA</t>
         </is>
       </c>
       <c r="B17" s="28" t="n"/>
@@ -1496,7 +1496,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>PRO MARTINEZ BRYAN</t>
+          <t>MARTINEZ BRYAN</t>
         </is>
       </c>
       <c r="B18" s="28" t="n"/>
@@ -1536,7 +1536,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>PRO VEGA NATALIA</t>
+          <t>VEGA NATALIA</t>
         </is>
       </c>
       <c r="B19" s="27" t="n"/>

</xml_diff>